<commit_message>
Translate database and workbook annotations
</commit_message>
<xml_diff>
--- a/Server/NewServer/bin/commonconfig/setting/circle_quest.xlsx
+++ b/Server/NewServer/bin/commonconfig/setting/circle_quest.xlsx
@@ -35,7 +35,7 @@
             <family val="3"/>
             <charset val="134"/>
           </rPr>
-          <t>作者:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -46,7 +46,7 @@
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
-标识任务池</t>
+Identifies the quest pool</t>
         </r>
       </text>
     </comment>
@@ -61,7 +61,7 @@
             <family val="3"/>
             <charset val="134"/>
           </rPr>
-          <t>作者:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -72,7 +72,7 @@
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
-同文档中</t>
+Same as the document's </t>
         </r>
         <r>
           <rPr>
@@ -91,7 +91,7 @@
             <family val="3"/>
             <charset val="134"/>
           </rPr>
-          <t>，标识组间互斥关系</t>
+          <t>; identifies mutually exclusive groups</t>
         </r>
       </text>
     </comment>
@@ -106,7 +106,7 @@
             <family val="3"/>
             <charset val="134"/>
           </rPr>
-          <t>作者:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -117,7 +117,7 @@
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
-每日大环可以完成的上限</t>
+Daily limit on completed quest cycles</t>
         </r>
       </text>
     </comment>
@@ -132,7 +132,7 @@
             <family val="3"/>
             <charset val="134"/>
           </rPr>
-          <t>作者:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -143,7 +143,7 @@
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
-奖励等级参考</t>
+Reward level reference</t>
         </r>
       </text>
     </comment>
@@ -158,7 +158,7 @@
             <family val="3"/>
             <charset val="134"/>
           </rPr>
-          <t>作者:</t>
+          <t>Author:</t>
         </r>
         <r>
           <rPr>
@@ -169,7 +169,7 @@
             <charset val="134"/>
           </rPr>
           <t xml:space="preserve">
-第几个大环</t>
+Quest cycle number</t>
         </r>
       </text>
     </comment>

</xml_diff>